<commit_message>
Perfect -> BC.Game | kl1m -> Envy
</commit_message>
<xml_diff>
--- a/file/history_updated.xlsx
+++ b/file/history_updated.xlsx
@@ -2665,7 +2665,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H18"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2695,65 +2695,65 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>1787536348426</v>
+        <v>1788874820852</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="str">
-        <v>RELEASED</v>
+        <v>FA SIGNING</v>
       </c>
       <c r="D2" t="str">
-        <v>fer</v>
+        <v>Perfecto</v>
       </c>
       <c r="E2" t="str">
-        <v>Lux Tenebris</v>
+        <v>Free Agency</v>
       </c>
       <c r="F2" t="str">
-        <v>Free Agency</v>
+        <v>BC.Game</v>
       </c>
       <c r="G2">
         <v>0</v>
       </c>
       <c r="H2" t="str">
-        <v>released to market for free</v>
+        <v>joined as Bench</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>1785396043745</v>
+        <v>1788874765369</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="str">
-        <v>PROMOTED</v>
+        <v>FA SIGNING</v>
       </c>
       <c r="D3" t="str">
-        <v>boltz</v>
+        <v>kl1m</v>
       </c>
       <c r="E3" t="str">
-        <v>Lux Tenebris</v>
+        <v>Free Agency</v>
       </c>
       <c r="F3" t="str">
-        <v>Lux Tenebris</v>
+        <v>Envy</v>
       </c>
       <c r="G3">
         <v>0</v>
       </c>
       <c r="H3" t="str">
-        <v>promoted to starter</v>
+        <v>joined as Bench</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>1785396042996</v>
+        <v>1787536348426</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" t="str">
-        <v>BENCHED</v>
+        <v>RELEASED</v>
       </c>
       <c r="D4" t="str">
         <v>fer</v>
@@ -2762,30 +2762,30 @@
         <v>Lux Tenebris</v>
       </c>
       <c r="F4" t="str">
-        <v>Lux Tenebris</v>
+        <v>Free Agency</v>
       </c>
       <c r="G4">
         <v>0</v>
       </c>
       <c r="H4" t="str">
-        <v>moved to bench</v>
+        <v>released to market for free</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>1785396011356</v>
+        <v>1785396043745</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" t="str">
-        <v>FA SIGNING</v>
+        <v>PROMOTED</v>
       </c>
       <c r="D5" t="str">
         <v>boltz</v>
       </c>
       <c r="E5" t="str">
-        <v>Free Agency</v>
+        <v>Lux Tenebris</v>
       </c>
       <c r="F5" t="str">
         <v>Lux Tenebris</v>
@@ -2794,64 +2794,64 @@
         <v>0</v>
       </c>
       <c r="H5" t="str">
-        <v>joined as Bench</v>
+        <v>promoted to starter</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>1783532394458</v>
+        <v>1785396042996</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
       <c r="C6" t="str">
-        <v>FA SIGNING</v>
+        <v>BENCHED</v>
       </c>
       <c r="D6" t="str">
-        <v>diskyb0b</v>
+        <v>fer</v>
       </c>
       <c r="E6" t="str">
-        <v>Free Agency</v>
+        <v>Lux Tenebris</v>
       </c>
       <c r="F6" t="str">
-        <v>Kappa Bar</v>
+        <v>Lux Tenebris</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
       <c r="H6" t="str">
-        <v>joined as Starter</v>
+        <v>moved to bench</v>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <v>1783532378345</v>
+        <v>1785396011356</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" t="str">
-        <v>TRANSFER</v>
+        <v>FA SIGNING</v>
       </c>
       <c r="D7" t="str">
-        <v>Gizmy</v>
+        <v>boltz</v>
       </c>
       <c r="E7" t="str">
-        <v>Kappa Bar</v>
+        <v>Free Agency</v>
       </c>
       <c r="F7" t="str">
-        <v>Iluminar</v>
+        <v>Lux Tenebris</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
       <c r="H7" t="str">
-        <v>CLAUSE DEAL · joined as Starter</v>
+        <v>joined as Bench</v>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <v>1783532335269</v>
+        <v>1783532394458</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -2860,13 +2860,13 @@
         <v>FA SIGNING</v>
       </c>
       <c r="D8" t="str">
-        <v>hades</v>
+        <v>diskyb0b</v>
       </c>
       <c r="E8" t="str">
         <v>Free Agency</v>
       </c>
       <c r="F8" t="str">
-        <v>Mythic</v>
+        <v>Kappa Bar</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -2877,7 +2877,7 @@
     </row>
     <row r="9">
       <c r="A9">
-        <v>1783532286477</v>
+        <v>1783532378345</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -2886,10 +2886,10 @@
         <v>TRANSFER</v>
       </c>
       <c r="D9" t="str">
-        <v>fl0m</v>
+        <v>Gizmy</v>
       </c>
       <c r="E9" t="str">
-        <v>Mythic</v>
+        <v>Kappa Bar</v>
       </c>
       <c r="F9" t="str">
         <v>Iluminar</v>
@@ -2903,7 +2903,7 @@
     </row>
     <row r="10">
       <c r="A10">
-        <v>1783531772696</v>
+        <v>1783532335269</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -2912,13 +2912,13 @@
         <v>FA SIGNING</v>
       </c>
       <c r="D10" t="str">
-        <v>taco</v>
+        <v>hades</v>
       </c>
       <c r="E10" t="str">
         <v>Free Agency</v>
       </c>
       <c r="F10" t="str">
-        <v>Lux Tenebris</v>
+        <v>Mythic</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -2929,33 +2929,33 @@
     </row>
     <row r="11">
       <c r="A11">
-        <v>1783531758984</v>
+        <v>1783532286477</v>
       </c>
       <c r="B11">
         <v>1</v>
       </c>
       <c r="C11" t="str">
-        <v>FA SIGNING</v>
+        <v>TRANSFER</v>
       </c>
       <c r="D11" t="str">
-        <v>fer</v>
+        <v>fl0m</v>
       </c>
       <c r="E11" t="str">
-        <v>Free Agency</v>
+        <v>Mythic</v>
       </c>
       <c r="F11" t="str">
-        <v>Lux Tenebris</v>
+        <v>Iluminar</v>
       </c>
       <c r="G11">
         <v>0</v>
       </c>
       <c r="H11" t="str">
-        <v>joined as Starter</v>
+        <v>CLAUSE DEAL · joined as Starter</v>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <v>1783531616692</v>
+        <v>1783531772696</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -2964,7 +2964,7 @@
         <v>FA SIGNING</v>
       </c>
       <c r="D12" t="str">
-        <v>kyourezz</v>
+        <v>taco</v>
       </c>
       <c r="E12" t="str">
         <v>Free Agency</v>
@@ -2981,118 +2981,170 @@
     </row>
     <row r="13">
       <c r="A13">
-        <v>1783531586211</v>
+        <v>1783531758984</v>
       </c>
       <c r="B13">
         <v>1</v>
       </c>
       <c r="C13" t="str">
-        <v>TRANSFER</v>
+        <v>FA SIGNING</v>
       </c>
       <c r="D13" t="str">
-        <v>heroghoxxt</v>
+        <v>fer</v>
       </c>
       <c r="E13" t="str">
-        <v>Iluminar</v>
+        <v>Free Agency</v>
       </c>
       <c r="F13" t="str">
         <v>Lux Tenebris</v>
       </c>
       <c r="G13">
-        <v>40000</v>
+        <v>0</v>
       </c>
       <c r="H13" t="str">
-        <v>CLAUSE DEAL · joined as Starter</v>
+        <v>joined as Starter</v>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <v>1783531583393</v>
+        <v>1783531616692</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="str">
-        <v>TRANSFER</v>
+        <v>FA SIGNING</v>
       </c>
       <c r="D14" t="str">
-        <v>kilzys</v>
+        <v>kyourezz</v>
       </c>
       <c r="E14" t="str">
-        <v>Iluminar</v>
+        <v>Free Agency</v>
       </c>
       <c r="F14" t="str">
         <v>Lux Tenebris</v>
       </c>
       <c r="G14">
-        <v>50000</v>
+        <v>0</v>
       </c>
       <c r="H14" t="str">
-        <v>CLAUSE DEAL · joined as Starter</v>
+        <v>joined as Starter</v>
       </c>
     </row>
     <row r="15">
       <c r="A15">
-        <v>1783473413103</v>
+        <v>1783531586211</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="str">
-        <v>FA SIGNING</v>
+        <v>TRANSFER</v>
       </c>
       <c r="D15" t="str">
-        <v>taco</v>
+        <v>heroghoxxt</v>
       </c>
       <c r="E15" t="str">
-        <v>Free Agency</v>
+        <v>Iluminar</v>
       </c>
       <c r="F15" t="str">
         <v>Lux Tenebris</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>40000</v>
       </c>
       <c r="H15" t="str">
-        <v>joined as Starter</v>
+        <v>CLAUSE DEAL · joined as Starter</v>
       </c>
     </row>
     <row r="16">
       <c r="A16">
-        <v>1783473388452</v>
+        <v>1783531583393</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" t="str">
-        <v>FA SIGNING</v>
+        <v>TRANSFER</v>
       </c>
       <c r="D16" t="str">
-        <v>fer</v>
+        <v>kilzys</v>
       </c>
       <c r="E16" t="str">
-        <v>Free Agency</v>
+        <v>Iluminar</v>
       </c>
       <c r="F16" t="str">
         <v>Lux Tenebris</v>
       </c>
       <c r="G16">
+        <v>50000</v>
+      </c>
+      <c r="H16" t="str">
+        <v>CLAUSE DEAL · joined as Starter</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>1783473413103</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17" t="str">
+        <v>FA SIGNING</v>
+      </c>
+      <c r="D17" t="str">
+        <v>taco</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Free Agency</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Lux Tenebris</v>
+      </c>
+      <c r="G17">
         <v>0</v>
       </c>
-      <c r="H16" t="str">
+      <c r="H17" t="str">
+        <v>joined as Starter</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>1783473388452</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18" t="str">
+        <v>FA SIGNING</v>
+      </c>
+      <c r="D18" t="str">
+        <v>fer</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Free Agency</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Lux Tenebris</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18" t="str">
         <v>joined as Starter</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H18"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3119,22 +3171,22 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>1787536347803</v>
+        <v>1788874820765</v>
       </c>
       <c r="B2" t="str">
-        <v>fer</v>
+        <v>Perfecto</v>
       </c>
       <c r="C2" t="str">
-        <v>—</v>
+        <v>BC.Game</v>
       </c>
       <c r="D2" t="str">
-        <v>Lux Tenebris</v>
+        <v>FREE AGENCY</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2" t="str">
-        <v>✅ RELEASED (FREE)</v>
+        <v>✅ FA SIGNING</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -3142,13 +3194,13 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>1785396010605</v>
+        <v>1788874765189</v>
       </c>
       <c r="B3" t="str">
-        <v>boltz</v>
+        <v>kl1m</v>
       </c>
       <c r="C3" t="str">
-        <v>Lux Tenebris</v>
+        <v>Envy</v>
       </c>
       <c r="D3" t="str">
         <v>FREE AGENCY</v>
@@ -3163,9 +3215,55 @@
         <v>1</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4">
+        <v>1787536347803</v>
+      </c>
+      <c r="B4" t="str">
+        <v>fer</v>
+      </c>
+      <c r="C4" t="str">
+        <v>—</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Lux Tenebris</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="str">
+        <v>✅ RELEASED (FREE)</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>1785396010605</v>
+      </c>
+      <c r="B5" t="str">
+        <v>boltz</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Lux Tenebris</v>
+      </c>
+      <c r="D5" t="str">
+        <v>FREE AGENCY</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" t="str">
+        <v>✅ FA SIGNING</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Big update - data
</commit_message>
<xml_diff>
--- a/file/history_updated.xlsx
+++ b/file/history_updated.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:M10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -420,16 +420,28 @@
         <v>scope</v>
       </c>
       <c r="F1" t="str">
+        <v>compRegion</v>
+      </c>
+      <c r="G1" t="str">
         <v>position</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>prizePool</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>wonAmount</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>month</v>
+      </c>
+      <c r="K1" t="str">
+        <v>kind</v>
+      </c>
+      <c r="L1" t="str">
+        <v>awardKey</v>
+      </c>
+      <c r="M1" t="str">
+        <v>note</v>
       </c>
     </row>
     <row r="2">
@@ -449,16 +461,28 @@
         <v>Regional</v>
       </c>
       <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
         <v>Third</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>1500</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>900</v>
       </c>
-      <c r="I2">
-        <v>1</v>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2" t="str">
+        <v>EVENT</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -478,16 +502,28 @@
         <v>Regional</v>
       </c>
       <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
         <v>Second</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>2000</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>1200</v>
       </c>
-      <c r="I3">
-        <v>1</v>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3" t="str">
+        <v>EVENT</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -507,16 +543,28 @@
         <v>Regional</v>
       </c>
       <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
         <v>Winner</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>3000</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>1800</v>
       </c>
-      <c r="I4">
-        <v>1</v>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4" t="str">
+        <v>EVENT</v>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -536,16 +584,28 @@
         <v>Regional</v>
       </c>
       <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
         <v>Third</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>1500</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>900</v>
       </c>
-      <c r="I5">
-        <v>1</v>
+      <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5" t="str">
+        <v>EVENT</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -565,16 +625,28 @@
         <v>Regional</v>
       </c>
       <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
         <v>Second</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>2000</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>1200</v>
       </c>
-      <c r="I6">
-        <v>1</v>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6" t="str">
+        <v>EVENT</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -594,16 +666,28 @@
         <v>Regional</v>
       </c>
       <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
         <v>Winner</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>3000</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>1800</v>
       </c>
-      <c r="I7">
-        <v>1</v>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="K7" t="str">
+        <v>EVENT</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -623,16 +707,28 @@
         <v>Global</v>
       </c>
       <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
         <v>Third</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>1790000</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>100000</v>
       </c>
-      <c r="I8">
-        <v>1</v>
+      <c r="J8">
+        <v>1</v>
+      </c>
+      <c r="K8" t="str">
+        <v>EVENT</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -652,16 +748,28 @@
         <v>Global</v>
       </c>
       <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
         <v>Second</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>1790000</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>170000</v>
       </c>
-      <c r="I9">
-        <v>1</v>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9" t="str">
+        <v>EVENT</v>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -681,28 +789,40 @@
         <v>Global</v>
       </c>
       <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
         <v>Winner</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <v>1790000</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>500000</v>
       </c>
-      <c r="I10">
-        <v>1</v>
+      <c r="J10">
+        <v>1</v>
+      </c>
+      <c r="K10" t="str">
+        <v>EVENT</v>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M10"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:M61"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -730,10 +850,19 @@
         <v>scope</v>
       </c>
       <c r="I1" t="str">
+        <v>compRegion</v>
+      </c>
+      <c r="J1" t="str">
         <v>position</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>month</v>
+      </c>
+      <c r="L1" t="str">
+        <v>awardKey</v>
+      </c>
+      <c r="M1" t="str">
+        <v>note</v>
       </c>
     </row>
     <row r="2">
@@ -762,10 +891,19 @@
         <v>Regional</v>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
         <v>Winner</v>
       </c>
-      <c r="J2">
-        <v>1</v>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -794,10 +932,19 @@
         <v>Regional</v>
       </c>
       <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
         <v>Winner</v>
       </c>
-      <c r="J3">
-        <v>1</v>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -826,10 +973,19 @@
         <v>Regional</v>
       </c>
       <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
         <v>Winner</v>
       </c>
-      <c r="J4">
-        <v>1</v>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -858,10 +1014,19 @@
         <v>Regional</v>
       </c>
       <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
         <v>Winner</v>
       </c>
-      <c r="J5">
-        <v>1</v>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -890,10 +1055,19 @@
         <v>Regional</v>
       </c>
       <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
         <v>Winner</v>
       </c>
-      <c r="J6">
-        <v>1</v>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -922,10 +1096,19 @@
         <v>Regional</v>
       </c>
       <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
         <v>Third</v>
       </c>
-      <c r="J7">
-        <v>1</v>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -954,10 +1137,19 @@
         <v>Regional</v>
       </c>
       <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
         <v>Third</v>
       </c>
-      <c r="J8">
-        <v>1</v>
+      <c r="K8">
+        <v>1</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -986,10 +1178,19 @@
         <v>Regional</v>
       </c>
       <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
         <v>Third</v>
       </c>
-      <c r="J9">
-        <v>1</v>
+      <c r="K9">
+        <v>1</v>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -1018,10 +1219,19 @@
         <v>Regional</v>
       </c>
       <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
         <v>Third</v>
       </c>
-      <c r="J10">
-        <v>1</v>
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -1050,10 +1260,19 @@
         <v>Regional</v>
       </c>
       <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
         <v>Third</v>
       </c>
-      <c r="J11">
-        <v>1</v>
+      <c r="K11">
+        <v>1</v>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -1082,10 +1301,19 @@
         <v>Regional</v>
       </c>
       <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
         <v>Second</v>
       </c>
-      <c r="J12">
-        <v>1</v>
+      <c r="K12">
+        <v>1</v>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -1114,10 +1342,19 @@
         <v>Regional</v>
       </c>
       <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
         <v>Second</v>
       </c>
-      <c r="J13">
-        <v>1</v>
+      <c r="K13">
+        <v>1</v>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -1146,10 +1383,19 @@
         <v>Regional</v>
       </c>
       <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
         <v>Second</v>
       </c>
-      <c r="J14">
-        <v>1</v>
+      <c r="K14">
+        <v>1</v>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -1178,10 +1424,19 @@
         <v>Regional</v>
       </c>
       <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
         <v>Second</v>
       </c>
-      <c r="J15">
-        <v>1</v>
+      <c r="K15">
+        <v>1</v>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -1210,10 +1465,19 @@
         <v>Regional</v>
       </c>
       <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
         <v>Second</v>
       </c>
-      <c r="J16">
-        <v>1</v>
+      <c r="K16">
+        <v>1</v>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -1242,10 +1506,19 @@
         <v>Regional</v>
       </c>
       <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
         <v>Winner</v>
       </c>
-      <c r="J17">
-        <v>1</v>
+      <c r="K17">
+        <v>1</v>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+      <c r="M17" t="str">
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -1274,10 +1547,19 @@
         <v>Regional</v>
       </c>
       <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
         <v>Winner</v>
       </c>
-      <c r="J18">
-        <v>1</v>
+      <c r="K18">
+        <v>1</v>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
+      <c r="M18" t="str">
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -1306,10 +1588,19 @@
         <v>Regional</v>
       </c>
       <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
         <v>Winner</v>
       </c>
-      <c r="J19">
-        <v>1</v>
+      <c r="K19">
+        <v>1</v>
+      </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
+      <c r="M19" t="str">
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -1338,10 +1629,19 @@
         <v>Regional</v>
       </c>
       <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
         <v>Winner</v>
       </c>
-      <c r="J20">
-        <v>1</v>
+      <c r="K20">
+        <v>1</v>
+      </c>
+      <c r="L20" t="str">
+        <v/>
+      </c>
+      <c r="M20" t="str">
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -1370,10 +1670,19 @@
         <v>Regional</v>
       </c>
       <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
         <v>Winner</v>
       </c>
-      <c r="J21">
-        <v>1</v>
+      <c r="K21">
+        <v>1</v>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+      <c r="M21" t="str">
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -1402,10 +1711,19 @@
         <v>Regional</v>
       </c>
       <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
         <v>Third</v>
       </c>
-      <c r="J22">
-        <v>1</v>
+      <c r="K22">
+        <v>1</v>
+      </c>
+      <c r="L22" t="str">
+        <v/>
+      </c>
+      <c r="M22" t="str">
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -1434,10 +1752,19 @@
         <v>Regional</v>
       </c>
       <c r="I23" t="str">
+        <v/>
+      </c>
+      <c r="J23" t="str">
         <v>Third</v>
       </c>
-      <c r="J23">
-        <v>1</v>
+      <c r="K23">
+        <v>1</v>
+      </c>
+      <c r="L23" t="str">
+        <v/>
+      </c>
+      <c r="M23" t="str">
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -1466,10 +1793,19 @@
         <v>Regional</v>
       </c>
       <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
         <v>Third</v>
       </c>
-      <c r="J24">
-        <v>1</v>
+      <c r="K24">
+        <v>1</v>
+      </c>
+      <c r="L24" t="str">
+        <v/>
+      </c>
+      <c r="M24" t="str">
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -1498,10 +1834,19 @@
         <v>Regional</v>
       </c>
       <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
         <v>Third</v>
       </c>
-      <c r="J25">
-        <v>1</v>
+      <c r="K25">
+        <v>1</v>
+      </c>
+      <c r="L25" t="str">
+        <v/>
+      </c>
+      <c r="M25" t="str">
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -1530,10 +1875,19 @@
         <v>Regional</v>
       </c>
       <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
         <v>Third</v>
       </c>
-      <c r="J26">
-        <v>1</v>
+      <c r="K26">
+        <v>1</v>
+      </c>
+      <c r="L26" t="str">
+        <v/>
+      </c>
+      <c r="M26" t="str">
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -1562,10 +1916,19 @@
         <v>Regional</v>
       </c>
       <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
         <v>Second</v>
       </c>
-      <c r="J27">
-        <v>1</v>
+      <c r="K27">
+        <v>1</v>
+      </c>
+      <c r="L27" t="str">
+        <v/>
+      </c>
+      <c r="M27" t="str">
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -1594,10 +1957,19 @@
         <v>Regional</v>
       </c>
       <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
         <v>Second</v>
       </c>
-      <c r="J28">
-        <v>1</v>
+      <c r="K28">
+        <v>1</v>
+      </c>
+      <c r="L28" t="str">
+        <v/>
+      </c>
+      <c r="M28" t="str">
+        <v/>
       </c>
     </row>
     <row r="29">
@@ -1626,10 +1998,19 @@
         <v>Regional</v>
       </c>
       <c r="I29" t="str">
+        <v/>
+      </c>
+      <c r="J29" t="str">
         <v>Second</v>
       </c>
-      <c r="J29">
-        <v>1</v>
+      <c r="K29">
+        <v>1</v>
+      </c>
+      <c r="L29" t="str">
+        <v/>
+      </c>
+      <c r="M29" t="str">
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -1658,10 +2039,19 @@
         <v>Regional</v>
       </c>
       <c r="I30" t="str">
+        <v/>
+      </c>
+      <c r="J30" t="str">
         <v>Second</v>
       </c>
-      <c r="J30">
-        <v>1</v>
+      <c r="K30">
+        <v>1</v>
+      </c>
+      <c r="L30" t="str">
+        <v/>
+      </c>
+      <c r="M30" t="str">
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -1690,10 +2080,19 @@
         <v>Regional</v>
       </c>
       <c r="I31" t="str">
+        <v/>
+      </c>
+      <c r="J31" t="str">
         <v>Second</v>
       </c>
-      <c r="J31">
-        <v>1</v>
+      <c r="K31">
+        <v>1</v>
+      </c>
+      <c r="L31" t="str">
+        <v/>
+      </c>
+      <c r="M31" t="str">
+        <v/>
       </c>
     </row>
     <row r="32">
@@ -1722,10 +2121,19 @@
         <v>Regional</v>
       </c>
       <c r="I32" t="str">
+        <v/>
+      </c>
+      <c r="J32" t="str">
         <v>Winner</v>
       </c>
-      <c r="J32">
-        <v>1</v>
+      <c r="K32">
+        <v>1</v>
+      </c>
+      <c r="L32" t="str">
+        <v/>
+      </c>
+      <c r="M32" t="str">
+        <v/>
       </c>
     </row>
     <row r="33">
@@ -1754,10 +2162,19 @@
         <v>Regional</v>
       </c>
       <c r="I33" t="str">
+        <v/>
+      </c>
+      <c r="J33" t="str">
         <v>Winner</v>
       </c>
-      <c r="J33">
-        <v>1</v>
+      <c r="K33">
+        <v>1</v>
+      </c>
+      <c r="L33" t="str">
+        <v/>
+      </c>
+      <c r="M33" t="str">
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -1786,10 +2203,19 @@
         <v>Regional</v>
       </c>
       <c r="I34" t="str">
+        <v/>
+      </c>
+      <c r="J34" t="str">
         <v>Winner</v>
       </c>
-      <c r="J34">
-        <v>1</v>
+      <c r="K34">
+        <v>1</v>
+      </c>
+      <c r="L34" t="str">
+        <v/>
+      </c>
+      <c r="M34" t="str">
+        <v/>
       </c>
     </row>
     <row r="35">
@@ -1818,10 +2244,19 @@
         <v>Regional</v>
       </c>
       <c r="I35" t="str">
+        <v/>
+      </c>
+      <c r="J35" t="str">
         <v>Winner</v>
       </c>
-      <c r="J35">
-        <v>1</v>
+      <c r="K35">
+        <v>1</v>
+      </c>
+      <c r="L35" t="str">
+        <v/>
+      </c>
+      <c r="M35" t="str">
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -1850,10 +2285,19 @@
         <v>Regional</v>
       </c>
       <c r="I36" t="str">
+        <v/>
+      </c>
+      <c r="J36" t="str">
         <v>Winner</v>
       </c>
-      <c r="J36">
-        <v>1</v>
+      <c r="K36">
+        <v>1</v>
+      </c>
+      <c r="L36" t="str">
+        <v/>
+      </c>
+      <c r="M36" t="str">
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -1882,10 +2326,19 @@
         <v>Regional</v>
       </c>
       <c r="I37" t="str">
+        <v/>
+      </c>
+      <c r="J37" t="str">
         <v>Second</v>
       </c>
-      <c r="J37">
-        <v>1</v>
+      <c r="K37">
+        <v>1</v>
+      </c>
+      <c r="L37" t="str">
+        <v/>
+      </c>
+      <c r="M37" t="str">
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -1914,10 +2367,19 @@
         <v>Regional</v>
       </c>
       <c r="I38" t="str">
+        <v/>
+      </c>
+      <c r="J38" t="str">
         <v>Second</v>
       </c>
-      <c r="J38">
-        <v>1</v>
+      <c r="K38">
+        <v>1</v>
+      </c>
+      <c r="L38" t="str">
+        <v/>
+      </c>
+      <c r="M38" t="str">
+        <v/>
       </c>
     </row>
     <row r="39">
@@ -1946,10 +2408,19 @@
         <v>Regional</v>
       </c>
       <c r="I39" t="str">
+        <v/>
+      </c>
+      <c r="J39" t="str">
         <v>Winner</v>
       </c>
-      <c r="J39">
-        <v>1</v>
+      <c r="K39">
+        <v>1</v>
+      </c>
+      <c r="L39" t="str">
+        <v/>
+      </c>
+      <c r="M39" t="str">
+        <v/>
       </c>
     </row>
     <row r="40">
@@ -1978,10 +2449,19 @@
         <v>Regional</v>
       </c>
       <c r="I40" t="str">
+        <v/>
+      </c>
+      <c r="J40" t="str">
         <v>Winner</v>
       </c>
-      <c r="J40">
-        <v>1</v>
+      <c r="K40">
+        <v>1</v>
+      </c>
+      <c r="L40" t="str">
+        <v/>
+      </c>
+      <c r="M40" t="str">
+        <v/>
       </c>
     </row>
     <row r="41">
@@ -2010,10 +2490,19 @@
         <v>Regional</v>
       </c>
       <c r="I41" t="str">
+        <v/>
+      </c>
+      <c r="J41" t="str">
         <v>Winner</v>
       </c>
-      <c r="J41">
-        <v>1</v>
+      <c r="K41">
+        <v>1</v>
+      </c>
+      <c r="L41" t="str">
+        <v/>
+      </c>
+      <c r="M41" t="str">
+        <v/>
       </c>
     </row>
     <row r="42">
@@ -2042,10 +2531,19 @@
         <v>Global</v>
       </c>
       <c r="I42" t="str">
+        <v/>
+      </c>
+      <c r="J42" t="str">
         <v>Third</v>
       </c>
-      <c r="J42">
-        <v>1</v>
+      <c r="K42">
+        <v>1</v>
+      </c>
+      <c r="L42" t="str">
+        <v/>
+      </c>
+      <c r="M42" t="str">
+        <v/>
       </c>
     </row>
     <row r="43">
@@ -2074,10 +2572,19 @@
         <v>Global</v>
       </c>
       <c r="I43" t="str">
+        <v/>
+      </c>
+      <c r="J43" t="str">
         <v>Second</v>
       </c>
-      <c r="J43">
-        <v>1</v>
+      <c r="K43">
+        <v>1</v>
+      </c>
+      <c r="L43" t="str">
+        <v/>
+      </c>
+      <c r="M43" t="str">
+        <v/>
       </c>
     </row>
     <row r="44">
@@ -2106,10 +2613,19 @@
         <v>Global</v>
       </c>
       <c r="I44" t="str">
+        <v/>
+      </c>
+      <c r="J44" t="str">
         <v>Second</v>
       </c>
-      <c r="J44">
-        <v>1</v>
+      <c r="K44">
+        <v>1</v>
+      </c>
+      <c r="L44" t="str">
+        <v/>
+      </c>
+      <c r="M44" t="str">
+        <v/>
       </c>
     </row>
     <row r="45">
@@ -2138,10 +2654,19 @@
         <v>Global</v>
       </c>
       <c r="I45" t="str">
+        <v/>
+      </c>
+      <c r="J45" t="str">
         <v>Winner</v>
       </c>
-      <c r="J45">
-        <v>1</v>
+      <c r="K45">
+        <v>1</v>
+      </c>
+      <c r="L45" t="str">
+        <v/>
+      </c>
+      <c r="M45" t="str">
+        <v/>
       </c>
     </row>
     <row r="46">
@@ -2170,10 +2695,19 @@
         <v>Global</v>
       </c>
       <c r="I46" t="str">
+        <v/>
+      </c>
+      <c r="J46" t="str">
         <v>Winner</v>
       </c>
-      <c r="J46">
-        <v>1</v>
+      <c r="K46">
+        <v>1</v>
+      </c>
+      <c r="L46" t="str">
+        <v/>
+      </c>
+      <c r="M46" t="str">
+        <v/>
       </c>
     </row>
     <row r="47">
@@ -2202,10 +2736,19 @@
         <v>Global</v>
       </c>
       <c r="I47" t="str">
+        <v/>
+      </c>
+      <c r="J47" t="str">
         <v>Third</v>
       </c>
-      <c r="J47">
-        <v>1</v>
+      <c r="K47">
+        <v>1</v>
+      </c>
+      <c r="L47" t="str">
+        <v/>
+      </c>
+      <c r="M47" t="str">
+        <v/>
       </c>
     </row>
     <row r="48">
@@ -2234,10 +2777,19 @@
         <v>Global</v>
       </c>
       <c r="I48" t="str">
+        <v/>
+      </c>
+      <c r="J48" t="str">
         <v>Third</v>
       </c>
-      <c r="J48">
-        <v>1</v>
+      <c r="K48">
+        <v>1</v>
+      </c>
+      <c r="L48" t="str">
+        <v/>
+      </c>
+      <c r="M48" t="str">
+        <v/>
       </c>
     </row>
     <row r="49">
@@ -2266,10 +2818,19 @@
         <v>Global</v>
       </c>
       <c r="I49" t="str">
+        <v/>
+      </c>
+      <c r="J49" t="str">
         <v>Third</v>
       </c>
-      <c r="J49">
-        <v>1</v>
+      <c r="K49">
+        <v>1</v>
+      </c>
+      <c r="L49" t="str">
+        <v/>
+      </c>
+      <c r="M49" t="str">
+        <v/>
       </c>
     </row>
     <row r="50">
@@ -2298,10 +2859,19 @@
         <v>Global</v>
       </c>
       <c r="I50" t="str">
+        <v/>
+      </c>
+      <c r="J50" t="str">
         <v>Third</v>
       </c>
-      <c r="J50">
-        <v>1</v>
+      <c r="K50">
+        <v>1</v>
+      </c>
+      <c r="L50" t="str">
+        <v/>
+      </c>
+      <c r="M50" t="str">
+        <v/>
       </c>
     </row>
     <row r="51">
@@ -2330,10 +2900,19 @@
         <v>Global</v>
       </c>
       <c r="I51" t="str">
+        <v/>
+      </c>
+      <c r="J51" t="str">
         <v>Third</v>
       </c>
-      <c r="J51">
-        <v>1</v>
+      <c r="K51">
+        <v>1</v>
+      </c>
+      <c r="L51" t="str">
+        <v/>
+      </c>
+      <c r="M51" t="str">
+        <v/>
       </c>
     </row>
     <row r="52">
@@ -2362,10 +2941,19 @@
         <v>Global</v>
       </c>
       <c r="I52" t="str">
+        <v/>
+      </c>
+      <c r="J52" t="str">
         <v>Second</v>
       </c>
-      <c r="J52">
-        <v>1</v>
+      <c r="K52">
+        <v>1</v>
+      </c>
+      <c r="L52" t="str">
+        <v/>
+      </c>
+      <c r="M52" t="str">
+        <v/>
       </c>
     </row>
     <row r="53">
@@ -2394,10 +2982,19 @@
         <v>Global</v>
       </c>
       <c r="I53" t="str">
+        <v/>
+      </c>
+      <c r="J53" t="str">
         <v>Second</v>
       </c>
-      <c r="J53">
-        <v>1</v>
+      <c r="K53">
+        <v>1</v>
+      </c>
+      <c r="L53" t="str">
+        <v/>
+      </c>
+      <c r="M53" t="str">
+        <v/>
       </c>
     </row>
     <row r="54">
@@ -2426,10 +3023,19 @@
         <v>Global</v>
       </c>
       <c r="I54" t="str">
+        <v/>
+      </c>
+      <c r="J54" t="str">
         <v>Second</v>
       </c>
-      <c r="J54">
-        <v>1</v>
+      <c r="K54">
+        <v>1</v>
+      </c>
+      <c r="L54" t="str">
+        <v/>
+      </c>
+      <c r="M54" t="str">
+        <v/>
       </c>
     </row>
     <row r="55">
@@ -2458,10 +3064,19 @@
         <v>Global</v>
       </c>
       <c r="I55" t="str">
+        <v/>
+      </c>
+      <c r="J55" t="str">
         <v>Second</v>
       </c>
-      <c r="J55">
-        <v>1</v>
+      <c r="K55">
+        <v>1</v>
+      </c>
+      <c r="L55" t="str">
+        <v/>
+      </c>
+      <c r="M55" t="str">
+        <v/>
       </c>
     </row>
     <row r="56">
@@ -2490,10 +3105,19 @@
         <v>Global</v>
       </c>
       <c r="I56" t="str">
+        <v/>
+      </c>
+      <c r="J56" t="str">
         <v>Second</v>
       </c>
-      <c r="J56">
-        <v>1</v>
+      <c r="K56">
+        <v>1</v>
+      </c>
+      <c r="L56" t="str">
+        <v/>
+      </c>
+      <c r="M56" t="str">
+        <v/>
       </c>
     </row>
     <row r="57">
@@ -2522,10 +3146,19 @@
         <v>Global</v>
       </c>
       <c r="I57" t="str">
+        <v/>
+      </c>
+      <c r="J57" t="str">
         <v>Winner</v>
       </c>
-      <c r="J57">
-        <v>1</v>
+      <c r="K57">
+        <v>1</v>
+      </c>
+      <c r="L57" t="str">
+        <v/>
+      </c>
+      <c r="M57" t="str">
+        <v/>
       </c>
     </row>
     <row r="58">
@@ -2554,10 +3187,19 @@
         <v>Global</v>
       </c>
       <c r="I58" t="str">
+        <v/>
+      </c>
+      <c r="J58" t="str">
         <v>Winner</v>
       </c>
-      <c r="J58">
-        <v>1</v>
+      <c r="K58">
+        <v>1</v>
+      </c>
+      <c r="L58" t="str">
+        <v/>
+      </c>
+      <c r="M58" t="str">
+        <v/>
       </c>
     </row>
     <row r="59">
@@ -2586,10 +3228,19 @@
         <v>Global</v>
       </c>
       <c r="I59" t="str">
+        <v/>
+      </c>
+      <c r="J59" t="str">
         <v>Winner</v>
       </c>
-      <c r="J59">
-        <v>1</v>
+      <c r="K59">
+        <v>1</v>
+      </c>
+      <c r="L59" t="str">
+        <v/>
+      </c>
+      <c r="M59" t="str">
+        <v/>
       </c>
     </row>
     <row r="60">
@@ -2618,10 +3269,19 @@
         <v>Global</v>
       </c>
       <c r="I60" t="str">
+        <v/>
+      </c>
+      <c r="J60" t="str">
         <v>Winner</v>
       </c>
-      <c r="J60">
-        <v>1</v>
+      <c r="K60">
+        <v>1</v>
+      </c>
+      <c r="L60" t="str">
+        <v/>
+      </c>
+      <c r="M60" t="str">
+        <v/>
       </c>
     </row>
     <row r="61">
@@ -2650,15 +3310,24 @@
         <v>Global</v>
       </c>
       <c r="I61" t="str">
+        <v/>
+      </c>
+      <c r="J61" t="str">
         <v>Winner</v>
       </c>
-      <c r="J61">
-        <v>1</v>
+      <c r="K61">
+        <v>1</v>
+      </c>
+      <c r="L61" t="str">
+        <v/>
+      </c>
+      <c r="M61" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M61"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>